<commit_message>
changes have been made
</commit_message>
<xml_diff>
--- a/Experiments data/K Size/K_Size_PGP_Graph.xlsx
+++ b/Experiments data/K Size/K_Size_PGP_Graph.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fengw\OneDrive\Documents\GitHub\KaMinPar_Java\Experiments data\K Size\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901B7AB9-C2A7-4617-BF87-53D43B707CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBE1FD6-8BC9-489B-96C7-3976265C143C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-210" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Edge Cuts" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="34">
   <si>
     <t>KaMinPar</t>
   </si>
@@ -329,17 +329,17 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -12535,7 +12535,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:R58"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
@@ -13324,7 +13324,7 @@
         <v>3.6779999999999999</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>22</v>
       </c>
@@ -13335,7 +13335,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="16"/>
     </row>
-    <row r="54" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="1" t="s">
         <v>6</v>
@@ -13361,21 +13361,8 @@
       <c r="I54" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N54" s="2"/>
-      <c r="O54" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="P54" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q54" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="R54" s="12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>2</v>
       </c>
@@ -13411,23 +13398,8 @@
         <f>AVERAGE(I4:I8)</f>
         <v>1.7050000000000001</v>
       </c>
-      <c r="N55" s="1">
-        <v>2</v>
-      </c>
-      <c r="O55">
-        <v>0.97059999999999991</v>
-      </c>
-      <c r="P55">
-        <v>1.1941999999999999</v>
-      </c>
-      <c r="Q55">
-        <v>1.7565999999999999</v>
-      </c>
-      <c r="R55">
-        <v>1.7050000000000001</v>
-      </c>
-    </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>4</v>
       </c>
@@ -13463,23 +13435,8 @@
         <f>AVERAGE(I14:I18)</f>
         <v>2.3527999999999998</v>
       </c>
-      <c r="N56" s="1">
-        <v>4</v>
-      </c>
-      <c r="O56">
-        <v>1.5190000000000001</v>
-      </c>
-      <c r="P56">
-        <v>1.4872000000000001</v>
-      </c>
-      <c r="Q56">
-        <v>2.4645999999999999</v>
-      </c>
-      <c r="R56">
-        <v>2.3527999999999998</v>
-      </c>
-    </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>8</v>
       </c>
@@ -13515,23 +13472,8 @@
         <f>AVERAGE(I24:I28)</f>
         <v>2.12</v>
       </c>
-      <c r="N57" s="1">
-        <v>8</v>
-      </c>
-      <c r="O57">
-        <v>2.0973999999999999</v>
-      </c>
-      <c r="P57">
-        <v>2.1905999999999999</v>
-      </c>
-      <c r="Q57">
-        <v>2.7736000000000001</v>
-      </c>
-      <c r="R57">
-        <v>2.12</v>
-      </c>
-    </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>16</v>
       </c>
@@ -13565,21 +13507,6 @@
       </c>
       <c r="I58">
         <f>AVERAGE(I35:I39)</f>
-        <v>3.3335999999999997</v>
-      </c>
-      <c r="N58" s="1">
-        <v>16</v>
-      </c>
-      <c r="O58">
-        <v>2.3555999999999999</v>
-      </c>
-      <c r="P58">
-        <v>2.7353999999999998</v>
-      </c>
-      <c r="Q58">
-        <v>3.4652000000000003</v>
-      </c>
-      <c r="R58">
         <v>3.3335999999999997</v>
       </c>
     </row>
@@ -13810,11 +13737,11 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
@@ -14288,15 +14215,15 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="20" t="s">
+      <c r="A47" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="20"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="19"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
@@ -14607,15 +14534,15 @@
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A66" s="20" t="s">
+      <c r="A66" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B66" s="20"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
-      <c r="E66" s="20"/>
-      <c r="F66" s="20"/>
-      <c r="G66" s="20"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="19"/>
+      <c r="E66" s="19"/>
+      <c r="F66" s="19"/>
+      <c r="G66" s="19"/>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="15" t="s">
@@ -15142,11 +15069,11 @@
       </c>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A95" s="17" t="s">
+      <c r="A95" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B95" s="17"/>
-      <c r="C95" s="17"/>
+      <c r="B95" s="20"/>
+      <c r="C95" s="20"/>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B96" s="1" t="s">
@@ -15261,6 +15188,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A86:G86"/>
+    <mergeCell ref="A87:G87"/>
+    <mergeCell ref="A95:C95"/>
+    <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A75:C75"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A11:C11"/>
@@ -15272,11 +15204,6 @@
     <mergeCell ref="A47:G47"/>
     <mergeCell ref="A48:G48"/>
     <mergeCell ref="A56:C56"/>
-    <mergeCell ref="A86:G86"/>
-    <mergeCell ref="A87:G87"/>
-    <mergeCell ref="A95:C95"/>
-    <mergeCell ref="A67:G67"/>
-    <mergeCell ref="A75:C75"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15688,15 +15615,15 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
@@ -15882,15 +15809,15 @@
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="20" t="s">
+      <c r="A38" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="20"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">

</xml_diff>